<commit_message>
Reject duplicate header names so RowData keys stay unambiguous.
Add 1-row schema and raw_header fixtures for duplicate header text on columns B and C.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/excel/testdata/raw_header/raw_header_tests.xlsx
+++ b/excel/testdata/raw_header/raw_header_tests.xlsx
@@ -11,15 +11,16 @@
     <sheet name="1-row-empty-header" sheetId="2" r:id="rId5"/>
     <sheet name="1-row-line-break" sheetId="3" r:id="rId6"/>
     <sheet name="1-row-horizontal-merge" sheetId="4" r:id="rId7"/>
-    <sheet name="2-row-simple" sheetId="5" r:id="rId8"/>
-    <sheet name="2-row-empty-cell" sheetId="6" r:id="rId9"/>
-    <sheet name="2-row-horizontal-merge" sheetId="7" r:id="rId10"/>
-    <sheet name="2-row-horizontal-merge-repeated" sheetId="8" r:id="rId11"/>
-    <sheet name="2-row-vertical-merge" sheetId="9" r:id="rId12"/>
-    <sheet name="2-row-vertical-merge-repeated" sheetId="10" r:id="rId13"/>
-    <sheet name="2-row-bidirectional-merge" sheetId="11" r:id="rId14"/>
-    <sheet name="2-row-bidirectional-merge-rep" sheetId="12" r:id="rId15"/>
-    <sheet name="2-row-mixed-merge" sheetId="13" r:id="rId16"/>
+    <sheet name="1-row-duplicate-header" sheetId="5" r:id="rId8"/>
+    <sheet name="2-row-simple" sheetId="6" r:id="rId9"/>
+    <sheet name="2-row-empty-cell" sheetId="7" r:id="rId10"/>
+    <sheet name="2-row-horizontal-merge" sheetId="8" r:id="rId11"/>
+    <sheet name="2-row-horizontal-merge-repeated" sheetId="9" r:id="rId12"/>
+    <sheet name="2-row-vertical-merge" sheetId="10" r:id="rId13"/>
+    <sheet name="2-row-vertical-merge-repeated" sheetId="11" r:id="rId14"/>
+    <sheet name="2-row-bidirectional-merge" sheetId="12" r:id="rId15"/>
+    <sheet name="2-row-bidirectional-merge-rep" sheetId="13" r:id="rId16"/>
+    <sheet name="2-row-mixed-merge" sheetId="14" r:id="rId17"/>
   </sheets>
   <calcPr calcId="122211"/>
 </workbook>
@@ -422,6 +423,36 @@
         <v>7</v>
       </c>
       <c r="C1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:A2"/>
+  </mergeCells>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
       <c r="D1" t="s">
@@ -445,7 +476,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1"/>
   <sheetData>
@@ -469,7 +500,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1"/>
   <sheetData>
@@ -501,7 +532,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1"/>
   <sheetData>
@@ -624,6 +655,25 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
         <v>6</v>
       </c>
       <c r="B1" t="s">
@@ -648,7 +698,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1"/>
   <sheetData>
@@ -675,7 +725,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1"/>
   <sheetData>
@@ -705,7 +755,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1"/>
   <sheetData>
@@ -749,34 +799,4 @@
     <mergeCell ref="D1:F1"/>
   </mergeCells>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="B2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:A2"/>
-  </mergeCells>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Add 2-row duplicate-header fixtures for resolved name collisions.
Columns B and C both map to group2 > headerB so schema tests cover multi-row naming plus rejectDuplicateHeaderNames.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/excel/testdata/raw_header/raw_header_tests.xlsx
+++ b/excel/testdata/raw_header/raw_header_tests.xlsx
@@ -13,14 +13,15 @@
     <sheet name="1-row-horizontal-merge" sheetId="4" r:id="rId7"/>
     <sheet name="1-row-duplicate-header" sheetId="5" r:id="rId8"/>
     <sheet name="2-row-simple" sheetId="6" r:id="rId9"/>
-    <sheet name="2-row-empty-cell" sheetId="7" r:id="rId10"/>
-    <sheet name="2-row-horizontal-merge" sheetId="8" r:id="rId11"/>
-    <sheet name="2-row-horizontal-merge-repeated" sheetId="9" r:id="rId12"/>
-    <sheet name="2-row-vertical-merge" sheetId="10" r:id="rId13"/>
-    <sheet name="2-row-vertical-merge-repeated" sheetId="11" r:id="rId14"/>
-    <sheet name="2-row-bidirectional-merge" sheetId="12" r:id="rId15"/>
-    <sheet name="2-row-bidirectional-merge-rep" sheetId="13" r:id="rId16"/>
-    <sheet name="2-row-mixed-merge" sheetId="14" r:id="rId17"/>
+    <sheet name="2-row-duplicate-header" sheetId="7" r:id="rId10"/>
+    <sheet name="2-row-empty-cell" sheetId="8" r:id="rId11"/>
+    <sheet name="2-row-horizontal-merge" sheetId="9" r:id="rId12"/>
+    <sheet name="2-row-horizontal-merge-repeated" sheetId="10" r:id="rId13"/>
+    <sheet name="2-row-vertical-merge" sheetId="11" r:id="rId14"/>
+    <sheet name="2-row-vertical-merge-repeated" sheetId="12" r:id="rId15"/>
+    <sheet name="2-row-bidirectional-merge" sheetId="13" r:id="rId16"/>
+    <sheet name="2-row-bidirectional-merge-rep" sheetId="14" r:id="rId17"/>
+    <sheet name="2-row-mixed-merge" sheetId="15" r:id="rId18"/>
   </sheets>
   <calcPr calcId="122211"/>
 </workbook>
@@ -417,6 +418,52 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="D1:F1"/>
+  </mergeCells>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
@@ -441,7 +488,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1"/>
   <sheetData>
@@ -476,7 +523,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1"/>
   <sheetData>
@@ -500,7 +547,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1"/>
   <sheetData>
@@ -532,7 +579,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1"/>
   <sheetData>
@@ -706,6 +753,36 @@
       <c r="A1" t="s">
         <v>6</v>
       </c>
+      <c r="B1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>6</v>
+      </c>
       <c r="C1" t="s">
         <v>8</v>
       </c>
@@ -725,7 +802,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1"/>
   <sheetData>
@@ -753,50 +830,4 @@
     <mergeCell ref="A1:B1"/>
   </mergeCells>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="D1:F1"/>
-  </mergeCells>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Add schema_header_3row fixtures including mixed merge layout.
Three-row header track covers simple and error cases plus a pass case with horizontal group merges and vertical leaf merges; data band spans A–H for mixed-merge.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/excel/testdata/raw_header/raw_header_tests.xlsx
+++ b/excel/testdata/raw_header/raw_header_tests.xlsx
@@ -22,13 +22,16 @@
     <sheet name="2-row-bidirectional-merge" sheetId="13" r:id="rId16"/>
     <sheet name="2-row-bidirectional-merge-rep" sheetId="14" r:id="rId17"/>
     <sheet name="2-row-mixed-merge" sheetId="15" r:id="rId18"/>
+    <sheet name="3-row-simple" sheetId="16" r:id="rId19"/>
+    <sheet name="3-row-bidirectional-merge" sheetId="17" r:id="rId20"/>
+    <sheet name="3-row-mixed-merge" sheetId="18" r:id="rId21"/>
   </sheets>
   <calcPr calcId="122211"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>headerA</t>
   </si>
@@ -91,6 +94,18 @@
   </si>
   <si>
     <t>headerK</t>
+  </si>
+  <si>
+    <t>subgroup1</t>
+  </si>
+  <si>
+    <t>subgroup2</t>
+  </si>
+  <si>
+    <t>subgroup3</t>
+  </si>
+  <si>
+    <t>tierA</t>
   </si>
 </sst>
 </file>
@@ -639,6 +654,139 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="C2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="C3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:B3"/>
+  </mergeCells>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G2" t="s">
+        <v>1</v>
+      </c>
+      <c r="H2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="F2:F3"/>
+    <mergeCell ref="G2:G3"/>
+    <mergeCell ref="H2:H3"/>
+  </mergeCells>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1"/>

</xml_diff>